<commit_message>
Auto update BMKG data
</commit_message>
<xml_diff>
--- a/data/data_suhu_lama.xlsx
+++ b/data/data_suhu_lama.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1970"/>
+  <dimension ref="A1:L1975"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83066,6 +83066,206 @@
         </is>
       </c>
     </row>
+    <row r="1971">
+      <c r="A1971" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1971" t="inlineStr">
+        <is>
+          <t>KEDIRI</t>
+        </is>
+      </c>
+      <c r="C1971" t="n">
+        <v>21</v>
+      </c>
+      <c r="D1971" t="n">
+        <v>32</v>
+      </c>
+      <c r="E1971" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F1971" t="n">
+        <v>73.45</v>
+      </c>
+      <c r="G1971" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H1971" t="inlineStr"/>
+      <c r="I1971" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="J1971" t="n">
+        <v>190</v>
+      </c>
+      <c r="K1971" t="n">
+        <v>13.82</v>
+      </c>
+      <c r="L1971" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1972" t="inlineStr">
+        <is>
+          <t>MALANG</t>
+        </is>
+      </c>
+      <c r="C1972" t="n">
+        <v>19</v>
+      </c>
+      <c r="D1972" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1972" t="n">
+        <v>24.35</v>
+      </c>
+      <c r="F1972" t="n">
+        <v>78.75</v>
+      </c>
+      <c r="G1972" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1972" t="inlineStr"/>
+      <c r="I1972" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="J1972" t="n">
+        <v>135</v>
+      </c>
+      <c r="K1972" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="L1972" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1973" t="inlineStr">
+        <is>
+          <t>PASURUAN</t>
+        </is>
+      </c>
+      <c r="C1973" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1973" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1973" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F1973" t="n">
+        <v>78.7</v>
+      </c>
+      <c r="G1973" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H1973" t="inlineStr"/>
+      <c r="I1973" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="J1973" t="n">
+        <v>67</v>
+      </c>
+      <c r="K1973" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="L1973" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1974" t="inlineStr">
+        <is>
+          <t>SIDOARJO</t>
+        </is>
+      </c>
+      <c r="C1974" t="n">
+        <v>24</v>
+      </c>
+      <c r="D1974" t="n">
+        <v>33</v>
+      </c>
+      <c r="E1974" t="n">
+        <v>28.65</v>
+      </c>
+      <c r="F1974" t="n">
+        <v>72.15000000000001</v>
+      </c>
+      <c r="G1974" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H1974" t="inlineStr"/>
+      <c r="I1974" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="J1974" t="n">
+        <v>92</v>
+      </c>
+      <c r="K1974" t="n">
+        <v>14.57</v>
+      </c>
+      <c r="L1974" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1975" t="inlineStr">
+        <is>
+          <t>SURABAYA</t>
+        </is>
+      </c>
+      <c r="C1975" t="n">
+        <v>24</v>
+      </c>
+      <c r="D1975" t="n">
+        <v>34</v>
+      </c>
+      <c r="E1975" t="n">
+        <v>28.65</v>
+      </c>
+      <c r="F1975" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="G1975" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H1975" t="inlineStr"/>
+      <c r="I1975" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J1975" t="n">
+        <v>109</v>
+      </c>
+      <c r="K1975" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="L1975" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>